<commit_message>
Replace real organisation profiles with BEFTA-only profiles across BEFTA definitions. Keep JSON and Excel definitions in sync.
</commit_message>
<xml_diff>
--- a/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_MASTER_GROUPACCESS.xlsx
+++ b/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_MASTER_GROUPACCESS.xlsx
@@ -2018,7 +2018,7 @@
     <t>GA_SOLICITOR</t>
   </si>
   <si>
-    <t>SOLICITOR_PROFILE</t>
+    <t>BEFTA_SOLICITOR_PROFILE</t>
   </si>
   <si>
     <t>BEFTA GA Solicitor Respondent for Org description</t>
@@ -2030,7 +2030,7 @@
     <t>GA_OGD</t>
   </si>
   <si>
-    <t>GOVERNMENT_ORGANISATION_PROFILE</t>
+    <t>BEFTA_GOVERNMENT_ORGANISATION_PROFILE</t>
   </si>
   <si>
     <t>BEFTA GA OGD Respondent for Org description2</t>

</xml_diff>